<commit_message>
truncamiento de los datos
</commit_message>
<xml_diff>
--- a/resultados_concordancia/resultados_numericos_concordancia.xlsx
+++ b/resultados_concordancia/resultados_numericos_concordancia.xlsx
@@ -218,7 +218,7 @@
     <t>LIMITE_SUPERIOR</t>
   </si>
   <si>
-    <t>Inf</t>
+    <t>30000</t>
   </si>
   <si>
     <t>C_TOLERANCIA_usuario</t>
@@ -622,10 +622,10 @@
         <v>16359</v>
       </c>
       <c r="C2">
-        <v>13498</v>
+        <v>13497</v>
       </c>
       <c r="D2">
-        <v>2861</v>
+        <v>2862</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -643,22 +643,22 @@
         <v>125</v>
       </c>
       <c r="J2">
-        <v>336.6063820189961</v>
+        <v>328.4399010515232</v>
       </c>
       <c r="K2">
-        <v>339.075</v>
+        <v>339</v>
       </c>
       <c r="L2">
-        <v>2678.520000000003</v>
+        <v>2667.871999999988</v>
       </c>
       <c r="M2">
-        <v>110559.6</v>
+        <v>15201.8</v>
       </c>
       <c r="N2">
-        <v>1115.321348129303</v>
+        <v>586.3160482779147</v>
       </c>
       <c r="O2">
-        <v>285.8778169014084</v>
+        <v>285.8028169014084</v>
       </c>
     </row>
     <row r="3" spans="1:15">
@@ -669,10 +669,10 @@
         <v>16359</v>
       </c>
       <c r="C3">
-        <v>13091</v>
+        <v>13090</v>
       </c>
       <c r="D3">
-        <v>3268</v>
+        <v>3269</v>
       </c>
       <c r="E3">
         <v>604</v>
@@ -681,31 +681,31 @@
         <v>-627.4</v>
       </c>
       <c r="G3">
-        <v>-119.42</v>
+        <v>-119.422</v>
       </c>
       <c r="H3">
         <v>40.4</v>
       </c>
       <c r="I3">
-        <v>123.333333333333</v>
+        <v>123.3205128205125</v>
       </c>
       <c r="J3">
-        <v>290.9279885250993</v>
+        <v>281.4523069352234</v>
       </c>
       <c r="K3">
-        <v>285.94</v>
+        <v>285.7958333333333</v>
       </c>
       <c r="L3">
-        <v>2321.440000000008</v>
+        <v>2318.510000000001</v>
       </c>
       <c r="M3">
-        <v>124327.6</v>
+        <v>11609.4</v>
       </c>
       <c r="N3">
-        <v>1199.866103213876</v>
+        <v>514.0788430622505</v>
       </c>
       <c r="O3">
-        <v>245.54</v>
+        <v>245.3958333333333</v>
       </c>
     </row>
     <row r="4" spans="1:15">
@@ -841,58 +841,58 @@
         <v>16</v>
       </c>
       <c r="D2">
-        <v>12966</v>
+        <v>12964</v>
       </c>
       <c r="E2">
-        <v>0.009639358436342692</v>
+        <v>0.02304880949229111</v>
       </c>
       <c r="F2">
-        <v>0.009614305205392163</v>
+        <v>0.02277533700928137</v>
       </c>
       <c r="G2">
-        <v>0.9974009441483085</v>
+        <v>0.9881350712234743</v>
       </c>
       <c r="H2">
-        <v>43.59755978480963</v>
+        <v>44.59641315719235</v>
       </c>
       <c r="I2">
-        <v>1646.54050614179</v>
+        <v>774.3319893482983</v>
       </c>
       <c r="J2">
-        <v>-3183.621832253098</v>
+        <v>-1473.094285965472</v>
       </c>
       <c r="K2">
-        <v>3270.816951822717</v>
+        <v>1562.287112279857</v>
       </c>
       <c r="L2">
-        <v>289.1545416134207</v>
+        <v>276.4262980296477</v>
       </c>
       <c r="M2">
-        <v>0.01025385021860633</v>
+        <v>0.0201966022829381</v>
       </c>
       <c r="N2">
-        <v>9.291723106429108E-05</v>
+        <v>0.0005312476190119292</v>
       </c>
       <c r="O2">
-        <v>1647.054125676733</v>
+        <v>775.5853398605492</v>
       </c>
       <c r="P2">
-        <v>411.9469172431915</v>
+        <v>393.9885212106773</v>
       </c>
       <c r="Q2">
-        <v>-0.007707611521305838</v>
+        <v>-0.01011957306808586</v>
       </c>
       <c r="R2">
-        <v>1133.242616315008</v>
+        <v>589.1519625184344</v>
       </c>
       <c r="S2" t="s">
         <v>40</v>
       </c>
       <c r="T2">
-        <v>0.9062162579052908</v>
+        <v>0.7999845726627584</v>
       </c>
       <c r="U2">
-        <v>0.5085570025452059</v>
+        <v>0.5525011816623022</v>
       </c>
     </row>
     <row r="3" spans="1:21">
@@ -906,58 +906,58 @@
         <v>17</v>
       </c>
       <c r="D3">
-        <v>13486</v>
+        <v>13485</v>
       </c>
       <c r="E3">
-        <v>0.1385015361346004</v>
+        <v>0.2693897963946854</v>
       </c>
       <c r="F3">
-        <v>0.08823318986161494</v>
+        <v>0.2430142579857595</v>
       </c>
       <c r="G3">
-        <v>0.6370556769555752</v>
+        <v>0.9020915462949354</v>
       </c>
       <c r="H3">
-        <v>153.5430107945261</v>
+        <v>145.3564288895053</v>
       </c>
       <c r="I3">
-        <v>1134.205928982306</v>
+        <v>618.5612987312616</v>
       </c>
       <c r="J3">
-        <v>-2069.500610010794</v>
+        <v>-1067.023716623768</v>
       </c>
       <c r="K3">
-        <v>2376.586631599847</v>
+        <v>1357.736574402778</v>
       </c>
       <c r="L3">
-        <v>166.1920741281014</v>
+        <v>121.4276676749639</v>
       </c>
       <c r="M3">
-        <v>0.05091358081561104</v>
+        <v>0.1883993118041931</v>
       </c>
       <c r="N3">
-        <v>0.01918267551164399</v>
+        <v>0.07257086240157005</v>
       </c>
       <c r="O3">
-        <v>1144.510006937811</v>
+        <v>635.3882262848159</v>
       </c>
       <c r="P3">
-        <v>265.922534148424</v>
+        <v>257.7442859121725</v>
       </c>
       <c r="Q3">
-        <v>0.000790009469400521</v>
+        <v>0.00206449603093551</v>
       </c>
       <c r="R3">
-        <v>1115.777728079267</v>
+        <v>586.5051064880641</v>
       </c>
       <c r="S3" t="s">
         <v>40</v>
       </c>
       <c r="T3">
-        <v>0.9475011122645707</v>
+        <v>0.8908416759362254</v>
       </c>
       <c r="U3">
-        <v>0.6703431650442255</v>
+        <v>0.643762961269421</v>
       </c>
     </row>
     <row r="4" spans="1:21">
@@ -971,58 +971,58 @@
         <v>17</v>
       </c>
       <c r="D4">
-        <v>13044</v>
+        <v>13043</v>
       </c>
       <c r="E4">
-        <v>0.04403345051252998</v>
+        <v>0.1077745016880416</v>
       </c>
       <c r="F4">
-        <v>0.02672111143668717</v>
+        <v>0.1026297130172764</v>
       </c>
       <c r="G4">
-        <v>0.6068366463601012</v>
+        <v>0.9522633963490075</v>
       </c>
       <c r="H4">
-        <v>110.6878798175715</v>
+        <v>101.1696008847967</v>
       </c>
       <c r="I4">
-        <v>1252.877368628629</v>
+        <v>622.8771234327759</v>
       </c>
       <c r="J4">
-        <v>-2344.95176269454</v>
+        <v>-1119.669561043444</v>
       </c>
       <c r="K4">
-        <v>2566.327522329684</v>
+        <v>1322.008762813037</v>
       </c>
       <c r="L4">
-        <v>176.3753365241506</v>
+        <v>156.5531872179095</v>
       </c>
       <c r="M4">
-        <v>0.01503057134810782</v>
+        <v>0.08587544551633608</v>
       </c>
       <c r="N4">
-        <v>0.001938944764039431</v>
+        <v>0.01161534321410574</v>
       </c>
       <c r="O4">
-        <v>1257.709492918298</v>
+        <v>631.0162067083221</v>
       </c>
       <c r="P4">
-        <v>315.7114595483427</v>
+        <v>306.2088996663791</v>
       </c>
       <c r="Q4">
-        <v>0.002896024572403214</v>
+        <v>0.02812125380559009</v>
       </c>
       <c r="R4">
-        <v>1201.995170789952</v>
+        <v>514.9415666426914</v>
       </c>
       <c r="S4" t="s">
         <v>40</v>
       </c>
       <c r="T4">
-        <v>0.9457988347132781</v>
+        <v>0.8298704285823814</v>
       </c>
       <c r="U4">
-        <v>0.6607536230413752</v>
+        <v>0.5854501954811441</v>
       </c>
     </row>
   </sheetData>
@@ -1065,7 +1065,7 @@
         <v>15</v>
       </c>
       <c r="C3">
-        <v>0.009639358436342692</v>
+        <v>0.02304880949229111</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1076,7 +1076,7 @@
         <v>15</v>
       </c>
       <c r="C4">
-        <v>0.1385015361346004</v>
+        <v>0.2693897963946853</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1087,7 +1087,7 @@
         <v>16</v>
       </c>
       <c r="C5">
-        <v>0.009639358436342692</v>
+        <v>0.02304880949229111</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1109,7 +1109,7 @@
         <v>16</v>
       </c>
       <c r="C7">
-        <v>0.04403345051252999</v>
+        <v>0.1077745016880416</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -1120,7 +1120,7 @@
         <v>17</v>
       </c>
       <c r="C8">
-        <v>0.1385015361346004</v>
+        <v>0.2693897963946853</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -1131,7 +1131,7 @@
         <v>17</v>
       </c>
       <c r="C9">
-        <v>0.04403345051252999</v>
+        <v>0.1077745016880416</v>
       </c>
     </row>
     <row r="10" spans="1:3">

</xml_diff>